<commit_message>
add RDK X5 category 180926
</commit_message>
<xml_diff>
--- a/data/cytron-tutorials-export.xlsx
+++ b/data/cytron-tutorials-export.xlsx
@@ -5694,7 +5694,11 @@
       <c r="C66" s="3" t="n">
         <v>46161</v>
       </c>
-      <c r="D66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E66" s="5" t="n">
         <v>620</v>
       </c>
@@ -5924,7 +5928,11 @@
       <c r="C69" s="3" t="n">
         <v>46155</v>
       </c>
-      <c r="D69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E69" s="5" t="n">
         <v>423</v>
       </c>
@@ -7288,7 +7296,11 @@
       <c r="C87" s="3" t="n">
         <v>46140</v>
       </c>
-      <c r="D87" s="4" t="inlineStr"/>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E87" s="5" t="n">
         <v>292</v>
       </c>
@@ -7436,7 +7448,11 @@
       <c r="C89" s="3" t="n">
         <v>46134</v>
       </c>
-      <c r="D89" s="4" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E89" s="5" t="n">
         <v>705</v>
       </c>
@@ -7834,7 +7850,11 @@
       <c r="C94" s="3" t="n">
         <v>46131</v>
       </c>
-      <c r="D94" s="4" t="inlineStr"/>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E94" s="5" t="n">
         <v>368</v>
       </c>
@@ -9786,7 +9806,7 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Other Controllers</t>
+          <t>Other Controllers, RDK X5</t>
         </is>
       </c>
       <c r="E119" s="5" t="n">
@@ -10638,7 +10658,11 @@
       <c r="C130" s="3" t="n">
         <v>46045</v>
       </c>
-      <c r="D130" s="4" t="inlineStr"/>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E130" s="5" t="n">
         <v>426</v>
       </c>
@@ -12400,7 +12424,11 @@
       <c r="C153" s="3" t="n">
         <v>45965</v>
       </c>
-      <c r="D153" s="4" t="inlineStr"/>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E153" s="5" t="n">
         <v>565</v>
       </c>
@@ -13436,7 +13464,7 @@
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>Other Controllers</t>
+          <t>Other Controllers, RDK X5</t>
         </is>
       </c>
       <c r="E166" s="5" t="n">
@@ -14762,7 +14790,7 @@
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>Other Controllers</t>
+          <t>Other Controllers, RDK X5</t>
         </is>
       </c>
       <c r="E183" s="5" t="n">
@@ -15622,7 +15650,11 @@
       <c r="C194" s="3" t="n">
         <v>45866</v>
       </c>
-      <c r="D194" s="4" t="inlineStr"/>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E194" s="5" t="n">
         <v>951</v>
       </c>
@@ -15696,7 +15728,11 @@
       <c r="C195" s="3" t="n">
         <v>45866</v>
       </c>
-      <c r="D195" s="4" t="inlineStr"/>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
       <c r="E195" s="5" t="n">
         <v>2775</v>
       </c>
@@ -74770,7 +74806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B74"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -74787,7 +74823,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Snapshot of https://my.cytron.io/tutorial taken 17 Sep 2026 — 932 posts.</t>
+          <t>Snapshot of https://my.cytron.io/tutorial taken 18 Sep 2026 — 932 posts.</t>
         </is>
       </c>
     </row>
@@ -75305,64 +75341,64 @@
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
+          <t>RDK X5</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
           <t>(no category)</t>
         </is>
       </c>
-      <c r="B58" s="9" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="B59" s="9" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
         <is>
           <t>Top 10 authors</t>
         </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="9" t="inlineStr">
-        <is>
-          <t>Idris Zainal Abidin</t>
-        </is>
-      </c>
-      <c r="B61" s="9" t="n">
-        <v>163</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>Abdulrahman Alhamed</t>
+          <t>Idris Zainal Abidin</t>
         </is>
       </c>
       <c r="B62" s="9" t="n">
-        <v>109</v>
+        <v>163</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>suadanwar</t>
+          <t>Abdulrahman Alhamed</t>
         </is>
       </c>
       <c r="B63" s="9" t="n">
-        <v>94</v>
+        <v>109</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>Khairul_Tajudin</t>
+          <t>suadanwar</t>
         </is>
       </c>
       <c r="B64" s="9" t="n">
-        <v>44</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>Hussien Jawhar Sathik</t>
+          <t>Khairul_Tajudin</t>
         </is>
       </c>
       <c r="B65" s="9" t="n">
@@ -75372,77 +75408,87 @@
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>Solehin Rizal</t>
+          <t>Hussien Jawhar Sathik</t>
         </is>
       </c>
       <c r="B66" s="9" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>Ober Choo</t>
+          <t>Solehin Rizal</t>
         </is>
       </c>
       <c r="B67" s="9" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>Asri Ruslan</t>
+          <t>Ober Choo</t>
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>Ebi Syakirin Aznan</t>
+          <t>Asri Ruslan</t>
         </is>
       </c>
       <c r="B69" s="9" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
+          <t>Ebi Syakirin Aznan</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
           <t>Rupa</t>
         </is>
       </c>
-      <c r="B70" s="9" t="n">
+      <c r="B71" s="9" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="10" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>Totals</t>
         </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="inlineStr">
-        <is>
-          <t>Total views</t>
-        </is>
-      </c>
-      <c r="B73" s="11" t="n">
-        <v>4904700</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
+          <t>Total views</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="n">
+        <v>4904700</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
           <t>Total likes</t>
         </is>
       </c>
-      <c r="B74" s="9" t="n">
+      <c r="B75" s="9" t="n">
         <v>280</v>
       </c>
     </row>
@@ -75484,7 +75530,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Every row was read from the public pages of https://my.cytron.io on 17 Sep 2026: the listing (/tutorial?page=N), each article page (/tutorial/slug) and the category search (/tutorial-search?categories=ID).</t>
+          <t>Every row was read from the public pages of https://my.cytron.io on 18 Sep 2026: the listing (/tutorial?page=N), each article page (/tutorial/slug) and the category search (/tutorial-search?categories=ID).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add RDK X5 / Robot Kits / ZOOM:BIT
</commit_message>
<xml_diff>
--- a/data/cytron-tutorials-export.xlsx
+++ b/data/cytron-tutorials-export.xlsx
@@ -782,7 +782,11 @@
       <c r="C4" s="3" t="n">
         <v>46282</v>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Robotics</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="n">
         <v>19</v>
       </c>
@@ -819,7 +823,11 @@
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Sumo Robot</t>
+        </is>
+      </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
           <t>https://my.cytron.io/tutorial/build-robot-sumo-500g-rc-mddrc5</t>
@@ -2252,7 +2260,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Robotics, Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
@@ -11412,7 +11420,7 @@
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>micro:bit, Robot Kits</t>
+          <t>micro:bit</t>
         </is>
       </c>
       <c r="E140" s="5" t="n">
@@ -11453,7 +11461,7 @@
       </c>
       <c r="M140" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>ZOOM:BIT</t>
         </is>
       </c>
       <c r="N140" s="7" t="inlineStr">
@@ -12545,7 +12553,7 @@
       </c>
       <c r="M154" s="4" t="inlineStr">
         <is>
-          <t>Edu:bit</t>
+          <t>EDU:BIT</t>
         </is>
       </c>
       <c r="N154" s="7" t="inlineStr">
@@ -13616,7 +13624,7 @@
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Components, Other Controllers, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics, Components, Other Controllers</t>
         </is>
       </c>
       <c r="E168" s="5" t="n">
@@ -13776,7 +13784,7 @@
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, Other Controllers, Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E170" s="5" t="n">
@@ -13815,11 +13823,7 @@
           <t>Beginner</t>
         </is>
       </c>
-      <c r="M170" s="4" t="inlineStr">
-        <is>
-          <t>Makers</t>
-        </is>
-      </c>
+      <c r="M170" s="4" t="inlineStr"/>
       <c r="N170" s="7" t="inlineStr">
         <is>
           <t>https://my.cytron.io/tutorial/robo-base-mini-obstacle-avoidance-robot-with-maker-uno-and-maker-drive</t>
@@ -15492,7 +15496,7 @@
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E192" s="5" t="n">
@@ -16112,7 +16116,7 @@
       </c>
       <c r="D200" s="4" t="inlineStr">
         <is>
-          <t>Robotics, Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E200" s="5" t="n">
@@ -16354,7 +16358,7 @@
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E203" s="5" t="n">
@@ -17068,7 +17072,7 @@
       </c>
       <c r="D212" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E212" s="5" t="n">
@@ -17540,7 +17544,7 @@
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Wireless &amp; IoT, Components, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics, Wireless &amp; IoT, Components</t>
         </is>
       </c>
       <c r="E218" s="5" t="n">
@@ -19436,7 +19440,7 @@
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, Wireless &amp; IoT, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics, Wireless &amp; IoT</t>
         </is>
       </c>
       <c r="E242" s="5" t="n">
@@ -20388,7 +20392,7 @@
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>Robotics, Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E254" s="5" t="n">
@@ -21082,7 +21086,7 @@
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E263" s="5" t="n">
@@ -21640,7 +21644,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>micro:bit, Robotics, Robot Kits</t>
+          <t>micro:bit, Robotics</t>
         </is>
       </c>
       <c r="E270" s="5" t="n">
@@ -21681,7 +21685,7 @@
       </c>
       <c r="M270" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit, Line Following Robot</t>
+          <t>REKA:BIT, Line Following Robot</t>
         </is>
       </c>
       <c r="N270" s="7" t="inlineStr">
@@ -21718,7 +21722,7 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E271" s="5" t="n">
@@ -21878,7 +21882,7 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics</t>
         </is>
       </c>
       <c r="E273" s="5" t="n">
@@ -22268,7 +22272,7 @@
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E278" s="5" t="n">
@@ -24374,7 +24378,7 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>micro:bit, Robot Kits</t>
+          <t>micro:bit, Robotics</t>
         </is>
       </c>
       <c r="E305" s="5" t="n">
@@ -25906,7 +25910,7 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>3D Modelling, Robot Kits</t>
+          <t>Robotics, 3D Modelling</t>
         </is>
       </c>
       <c r="E325" s="5" t="n">
@@ -26218,7 +26222,7 @@
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Robotics, 3D Modelling, Robot Kits</t>
+          <t>Robotics, 3D Modelling</t>
         </is>
       </c>
       <c r="E329" s="5" t="n">
@@ -26768,7 +26772,7 @@
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E336" s="5" t="n">
@@ -28102,7 +28106,7 @@
       </c>
       <c r="D353" s="4" t="inlineStr">
         <is>
-          <t>Robotics, Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E353" s="5" t="n">
@@ -28878,7 +28882,7 @@
       </c>
       <c r="D363" s="4" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E363" s="5" t="n">
@@ -29506,7 +29510,7 @@
       </c>
       <c r="D371" s="4" t="inlineStr">
         <is>
-          <t>Robotics, Robot Kits</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E371" s="5" t="n">
@@ -29588,7 +29592,7 @@
       </c>
       <c r="D372" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics</t>
         </is>
       </c>
       <c r="E372" s="5" t="n">
@@ -31164,7 +31168,7 @@
       </c>
       <c r="D392" s="4" t="inlineStr">
         <is>
-          <t>Robotics, 3D Modelling, Robot Kits</t>
+          <t>Robotics, 3D Modelling</t>
         </is>
       </c>
       <c r="E392" s="5" t="n">
@@ -31562,7 +31566,7 @@
       </c>
       <c r="D397" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, 3D Modelling, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics, 3D Modelling</t>
         </is>
       </c>
       <c r="E397" s="5" t="n">
@@ -35718,7 +35722,7 @@
       </c>
       <c r="D451" s="4" t="inlineStr">
         <is>
-          <t>Raspberry Pi, Robot Kits</t>
+          <t>Raspberry Pi, Robotics</t>
         </is>
       </c>
       <c r="E451" s="5" t="n">
@@ -36527,7 +36531,7 @@
       <c r="L461" s="4" t="inlineStr"/>
       <c r="M461" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>REKA:BIT</t>
         </is>
       </c>
       <c r="N461" s="7" t="inlineStr">
@@ -37619,7 +37623,7 @@
       </c>
       <c r="M475" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>REKA:BIT</t>
         </is>
       </c>
       <c r="N475" s="7" t="inlineStr">
@@ -40551,7 +40555,7 @@
       </c>
       <c r="M513" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>REKA:BIT</t>
         </is>
       </c>
       <c r="N513" s="7" t="inlineStr">
@@ -41694,7 +41698,7 @@
       </c>
       <c r="D528" s="4" t="inlineStr">
         <is>
-          <t>Raspberry Pi, Robotics, Robot Kits</t>
+          <t>Raspberry Pi, Robotics</t>
         </is>
       </c>
       <c r="E528" s="5" t="n">
@@ -44213,7 +44217,7 @@
       </c>
       <c r="D560" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, 3D Modelling, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics, 3D Modelling</t>
         </is>
       </c>
       <c r="E560" s="5" t="n">
@@ -47412,7 +47416,7 @@
       </c>
       <c r="M600" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>REKA:BIT</t>
         </is>
       </c>
       <c r="N600" s="7" t="inlineStr">
@@ -48057,7 +48061,7 @@
       </c>
       <c r="M608" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>REKA:BIT</t>
         </is>
       </c>
       <c r="N608" s="7" t="inlineStr">
@@ -49427,7 +49431,7 @@
       </c>
       <c r="M625" s="4" t="inlineStr">
         <is>
-          <t>Reka:bit</t>
+          <t>REKA:BIT</t>
         </is>
       </c>
       <c r="N625" s="7" t="inlineStr">
@@ -57313,7 +57317,7 @@
       </c>
       <c r="M724" s="4" t="inlineStr">
         <is>
-          <t>Edu:bit</t>
+          <t>EDU:BIT</t>
         </is>
       </c>
       <c r="N724" s="7" t="inlineStr">
@@ -58306,7 +58310,7 @@
       </c>
       <c r="D737" s="4" t="inlineStr">
         <is>
-          <t>Raspberry Pi, Robotics, Other Controllers, Robot Kits</t>
+          <t>Raspberry Pi, Robotics, Other Controllers</t>
         </is>
       </c>
       <c r="E737" s="5" t="n">
@@ -62509,7 +62513,7 @@
       <c r="L790" s="4" t="inlineStr"/>
       <c r="M790" s="4" t="inlineStr">
         <is>
-          <t>Edu:bit</t>
+          <t>EDU:BIT</t>
         </is>
       </c>
       <c r="N790" s="7" t="inlineStr">
@@ -62911,7 +62915,7 @@
       </c>
       <c r="M795" s="4" t="inlineStr">
         <is>
-          <t>Edu:bit</t>
+          <t>EDU:BIT</t>
         </is>
       </c>
       <c r="N795" s="7" t="inlineStr">
@@ -63149,7 +63153,7 @@
       </c>
       <c r="M798" s="4" t="inlineStr">
         <is>
-          <t>Edu:bit</t>
+          <t>EDU:BIT</t>
         </is>
       </c>
       <c r="N798" s="7" t="inlineStr">
@@ -68664,7 +68668,7 @@
       </c>
       <c r="D868" s="4" t="inlineStr">
         <is>
-          <t>Robotics, Components, Robot Kits</t>
+          <t>Robotics, Components</t>
         </is>
       </c>
       <c r="E868" s="5" t="n">
@@ -72509,7 +72513,7 @@
       </c>
       <c r="D917" s="4" t="inlineStr">
         <is>
-          <t>Arduino Ecosystem, Robotics, Robot Kits</t>
+          <t>Arduino Ecosystem, Robotics</t>
         </is>
       </c>
       <c r="E917" s="5" t="n">
@@ -74965,7 +74969,7 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21">
@@ -75015,7 +75019,7 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26">
@@ -75025,7 +75029,7 @@
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27">
@@ -75161,17 +75165,17 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Reka:bit</t>
+          <t xml:space="preserve">    REKA:BIT</t>
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Edu:bit</t>
+          <t xml:space="preserve">    EDU:BIT</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
@@ -75191,11 +75195,11 @@
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>3D Modelling</t>
+          <t xml:space="preserve">    ZOOM:BIT</t>
         </is>
       </c>
       <c r="B43" s="9" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -75205,7 +75209,7 @@
         </is>
       </c>
       <c r="B44" s="9" t="n">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45">
@@ -75221,121 +75225,121 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    rero</t>
+          <t xml:space="preserve">    Sumo Robot</t>
         </is>
       </c>
       <c r="B46" s="9" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>NVIDIA AI</t>
+          <t xml:space="preserve">    Line Following Robot</t>
         </is>
       </c>
       <c r="B47" s="9" t="n">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Jetson Orin NX</t>
+          <t xml:space="preserve">    Soccer Robot</t>
         </is>
       </c>
       <c r="B48" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Jetson Nano</t>
+          <t xml:space="preserve">    Battle Robot</t>
         </is>
       </c>
       <c r="B49" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>Miscellaneous</t>
+          <t xml:space="preserve">    rero</t>
         </is>
       </c>
       <c r="B50" s="9" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    News</t>
+          <t>3D Modelling</t>
         </is>
       </c>
       <c r="B51" s="9" t="n">
-        <v>33</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Seminars &amp; Workshop</t>
+          <t>NVIDIA AI</t>
         </is>
       </c>
       <c r="B52" s="9" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>Robot Kits</t>
+          <t xml:space="preserve">    Jetson Orin NX</t>
         </is>
       </c>
       <c r="B53" s="9" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Line Following Robot</t>
+          <t xml:space="preserve">    Jetson Nano</t>
         </is>
       </c>
       <c r="B54" s="9" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Sumo Robot</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="B55" s="9" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Soccer Robot</t>
+          <t xml:space="preserve">    News</t>
         </is>
       </c>
       <c r="B56" s="9" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Battle Robot</t>
+          <t xml:space="preserve">    Seminars &amp; Workshop</t>
         </is>
       </c>
       <c r="B57" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58">
@@ -75355,7 +75359,7 @@
         </is>
       </c>
       <c r="B59" s="9" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="61">

</xml_diff>

<commit_message>
Other Controllers fix to GitHub Pages
</commit_message>
<xml_diff>
--- a/data/cytron-tutorials-export.xlsx
+++ b/data/cytron-tutorials-export.xlsx
@@ -75019,7 +75019,7 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26">
@@ -75045,21 +75045,21 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    PIC Microcontroller</t>
+          <t xml:space="preserve">    Teensy</t>
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Teensy</t>
+          <t xml:space="preserve">    PIC Microcontroller</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">

</xml_diff>